<commit_message>
Add NRCS school + multi-school architecture, cross-school conflict check
- model.py: SchoolConfig system; NRHS & NRCS configs; dedicated loaders for each
  (NRHS class-row allotment / label-row P1; NRCS subject-row allotment / Day-Period P1)
- solver/verify/writer/pdf/audit now read rules from m.cfg (school-agnostic)
- NRCS rules: Sonu afternoon; Gowtham/Sunita/Riya/Bheema morning; Karate Thu P6;
  P.E.T P5-7; Oral pinned P1 (LKG); Phy/Che + Eng Gram inheritance; Class 10 no study hour
- solver: minimal morning-window relaxation (P5) with precise reporting when a class
  is morning-overloaded (NRCS Class 9)
- cross_check.py: flags shared-teacher clashes across schools (Lalitha 23x)
- dashboard: School selector (NRHS/NRCS); all features per-school; PDF/xlsx names per school
- NRCS OPTIMAL, 0 hard violations, audit 504/504 PASS; NRHS unchanged 588/588 PASS

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NRHS/Output/NRHS_Timetable_Final.xlsx
+++ b/NRHS/Output/NRHS_Timetable_Final.xlsx
@@ -701,7 +701,7 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>UKG (A) (ENG)</t>
+          <t>UKG (A) (MATH)</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
@@ -896,7 +896,7 @@
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>UKG (A) (MATH)</t>
+          <t>UKG (A) (ENG)</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -1026,7 +1026,11 @@
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr"/>
-      <c r="C16" s="7" t="inlineStr"/>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Class 8 (BIO)</t>
+        </is>
+      </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
           <t>Class 10 (BIO)</t>
@@ -1072,11 +1076,7 @@
           <t>Class 10 (BIO)</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
-        <is>
-          <t>Class 8 (BIO)</t>
-        </is>
-      </c>
+      <c r="C18" s="7" t="inlineStr"/>
       <c r="D18" s="7" t="inlineStr">
         <is>
           <t>Class 9 (BIO)</t>
@@ -1099,12 +1099,12 @@
           <t>Class 8 (BIO)</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr"/>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>Class 9 (BIO)</t>
         </is>
       </c>
+      <c r="D19" s="7" t="inlineStr"/>
       <c r="E19" s="7" t="inlineStr"/>
       <c r="F19" s="7" t="inlineStr"/>
       <c r="G19" s="7" t="inlineStr"/>
@@ -1192,12 +1192,12 @@
       <c r="D23" s="7" t="inlineStr"/>
       <c r="E23" s="7" t="inlineStr">
         <is>
+          <t>Class 5 (MATH)</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
           <t>Class 4 (MATH)</t>
-        </is>
-      </c>
-      <c r="F23" s="7" t="inlineStr">
-        <is>
-          <t>Class 5 (MATH)</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr"/>
@@ -1265,12 +1265,12 @@
       <c r="C25" s="7" t="inlineStr"/>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>Class 6 (MATH)</t>
+          <t>Class 5 (MATH)</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>Class 5 (MATH)</t>
+          <t>Class 4 (MATH)</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
@@ -1281,7 +1281,7 @@
       <c r="G25" s="7" t="inlineStr"/>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>Class 4 (MATH)</t>
+          <t>Class 6 (MATH)</t>
         </is>
       </c>
       <c r="I25" s="8" t="inlineStr">
@@ -1381,13 +1381,13 @@
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Class 4 (MATH)</t>
+          <t>Class 6 (MATH)</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr"/>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>Class 5 (MATH)</t>
+          <t>Class 4 (MATH)</t>
         </is>
       </c>
       <c r="F28" s="7" t="inlineStr">
@@ -1398,7 +1398,7 @@
       <c r="G28" s="7" t="inlineStr"/>
       <c r="H28" s="7" t="inlineStr">
         <is>
-          <t>Class 6 (MATH)</t>
+          <t>Class 5 (MATH)</t>
         </is>
       </c>
       <c r="I28" s="8" t="inlineStr">
@@ -1477,12 +1477,12 @@
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
+          <t>Class 1(A) (TEL)</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
           <t>Class 1(A) (MATH)</t>
-        </is>
-      </c>
-      <c r="C32" s="7" t="inlineStr">
-        <is>
-          <t>Class 1(A) (TEL)</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
@@ -1525,7 +1525,7 @@
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Class 1(A) (HIN)</t>
+          <t>Class 1(A) (MATH)</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
@@ -1536,7 +1536,7 @@
       <c r="E33" s="7" t="inlineStr"/>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>Class 1(A) (MATH)</t>
+          <t>Class 1(A) (G.K)</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
@@ -1588,7 +1588,7 @@
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>Class 1(A) (G.K)</t>
+          <t>Class 2 (MATH)</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr">
@@ -1610,27 +1610,27 @@
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
+          <t>Class 1(A) (EVS)</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Class 1(A) (ENG)</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>Class 1(A) (TEL)</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>Class 1(A) (HIN)</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
           <t>Class 1(A) (MATH)</t>
-        </is>
-      </c>
-      <c r="C35" s="7" t="inlineStr">
-        <is>
-          <t>Class 1(A) (ENG)</t>
-        </is>
-      </c>
-      <c r="D35" s="7" t="inlineStr">
-        <is>
-          <t>Class 1(A) (TEL)</t>
-        </is>
-      </c>
-      <c r="E35" s="7" t="inlineStr">
-        <is>
-          <t>Class 1(A) (HIN)</t>
-        </is>
-      </c>
-      <c r="F35" s="7" t="inlineStr">
-        <is>
-          <t>Class 1(A) (EVS)</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>Class 1(A) (ENG)</t>
+          <t>Class 1(A) (HIN)</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr">
@@ -1700,32 +1700,32 @@
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
+          <t>Class 1(A) (ENG)</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Class 1(A) (ENG)</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>Class 1(A) (MATH)</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
           <t>Class 1(A) (TEL)</t>
         </is>
       </c>
-      <c r="C37" s="7" t="inlineStr">
-        <is>
-          <t>Class 1(A) (ENG)</t>
-        </is>
-      </c>
-      <c r="D37" s="7" t="inlineStr">
-        <is>
-          <t>Class 1(A) (MATH)</t>
-        </is>
-      </c>
-      <c r="E37" s="7" t="inlineStr">
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>Class 1(A) (HIN)</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="inlineStr">
         <is>
           <t>Class 1(A) (EVS)</t>
-        </is>
-      </c>
-      <c r="F37" s="7" t="inlineStr">
-        <is>
-          <t>Class 1(A) (HIN)</t>
-        </is>
-      </c>
-      <c r="G37" s="7" t="inlineStr">
-        <is>
-          <t>Class 2 (MATH)</t>
         </is>
       </c>
       <c r="H37" s="7" t="inlineStr">
@@ -2298,12 +2298,12 @@
       </c>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>Class 7 (PHY)</t>
+          <t>Class 7 (CHEM)</t>
         </is>
       </c>
       <c r="H59" s="7" t="inlineStr">
         <is>
-          <t>Class 7 (CHEM)</t>
+          <t>Class 6 (CHEM)</t>
         </is>
       </c>
       <c r="I59" s="8" t="inlineStr">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>Class 7 (G.K)</t>
+          <t>Class 7 (PHY)</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr"/>
@@ -2341,7 +2341,7 @@
       </c>
       <c r="G60" s="7" t="inlineStr">
         <is>
-          <t>Class 7 (CHEM)</t>
+          <t>Class 7 (G.K)</t>
         </is>
       </c>
       <c r="H60" s="7" t="inlineStr"/>
@@ -2381,7 +2381,7 @@
       <c r="G61" s="7" t="inlineStr"/>
       <c r="H61" s="7" t="inlineStr">
         <is>
-          <t>Class 7 (PHY)</t>
+          <t>Class 7 (CHEM)</t>
         </is>
       </c>
       <c r="I61" s="8" t="inlineStr">
@@ -2399,7 +2399,7 @@
       <c r="B62" s="7" t="inlineStr"/>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>Class 6 (CHEM)</t>
+          <t>Class 6 (PHY)</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
@@ -2491,7 +2491,7 @@
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>Class 6 (PHY)</t>
+          <t>Class 7 (PHY)</t>
         </is>
       </c>
       <c r="F64" s="7" t="inlineStr">
@@ -2772,13 +2772,13 @@
       </c>
       <c r="F73" s="7" t="inlineStr">
         <is>
-          <t>Class 6 (TEL)</t>
+          <t>Class 7 (TEL)</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr"/>
       <c r="H73" s="7" t="inlineStr">
         <is>
-          <t>Class 7 (TEL)</t>
+          <t>Class 6 (TEL)</t>
         </is>
       </c>
       <c r="I73" s="7" t="inlineStr"/>
@@ -2853,7 +2853,7 @@
       </c>
       <c r="B77" s="7" t="inlineStr">
         <is>
-          <t>UKG (B) (EVS)</t>
+          <t>UKG (B) (ENG)</t>
         </is>
       </c>
       <c r="C77" s="7" t="inlineStr">
@@ -2923,11 +2923,7 @@
           <t>UKG (B) (MATH)</t>
         </is>
       </c>
-      <c r="G78" s="7" t="inlineStr">
-        <is>
-          <t>UKG (B) (ENG)</t>
-        </is>
-      </c>
+      <c r="G78" s="7" t="inlineStr"/>
       <c r="H78" s="7" t="inlineStr">
         <is>
           <t>UKG (B) (MATH)</t>
@@ -3060,7 +3056,11 @@
           <t>UKG (B) (TEL)</t>
         </is>
       </c>
-      <c r="G81" s="7" t="inlineStr"/>
+      <c r="G81" s="7" t="inlineStr">
+        <is>
+          <t>UKG (B) (EVS)</t>
+        </is>
+      </c>
       <c r="H81" s="7" t="inlineStr">
         <is>
           <t>UKG (B) (EVS)</t>
@@ -3190,13 +3190,13 @@
       </c>
       <c r="C86" s="7" t="inlineStr">
         <is>
-          <t>Class 4 (ENG)</t>
+          <t>Class 3 (ENG)</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr"/>
       <c r="E86" s="7" t="inlineStr">
         <is>
-          <t>Class 5 (ENG)</t>
+          <t>Class 4 (ENG)</t>
         </is>
       </c>
       <c r="F86" s="7" t="inlineStr">
@@ -3204,12 +3204,12 @@
           <t>Class 6 (ENG)</t>
         </is>
       </c>
-      <c r="G86" s="7" t="inlineStr">
-        <is>
-          <t>Class 3 (ENG)</t>
-        </is>
-      </c>
-      <c r="H86" s="7" t="inlineStr"/>
+      <c r="G86" s="7" t="inlineStr"/>
+      <c r="H86" s="7" t="inlineStr">
+        <is>
+          <t>Class 4 (ENG)</t>
+        </is>
+      </c>
       <c r="I86" s="8" t="inlineStr">
         <is>
           <t>Class 3</t>
@@ -3234,7 +3234,7 @@
       </c>
       <c r="D87" s="7" t="inlineStr">
         <is>
-          <t>Class 4 (ENG)</t>
+          <t>Class 5 (ENG)</t>
         </is>
       </c>
       <c r="E87" s="7" t="inlineStr"/>
@@ -3402,7 +3402,7 @@
       </c>
       <c r="D91" s="7" t="inlineStr">
         <is>
-          <t>Class 6 (ENG)</t>
+          <t>Class 5 (ENG)</t>
         </is>
       </c>
       <c r="E91" s="7" t="inlineStr"/>
@@ -3413,7 +3413,7 @@
       </c>
       <c r="G91" s="7" t="inlineStr">
         <is>
-          <t>Class 5 (ENG)</t>
+          <t>Class 6 (ENG)</t>
         </is>
       </c>
       <c r="H91" s="7" t="inlineStr">
@@ -3502,7 +3502,7 @@
       </c>
       <c r="C95" s="7" t="inlineStr">
         <is>
-          <t>Class 3 (TEL)</t>
+          <t>Class 4 (TEL)</t>
         </is>
       </c>
       <c r="D95" s="7" t="inlineStr"/>
@@ -3513,12 +3513,12 @@
       </c>
       <c r="F95" s="7" t="inlineStr">
         <is>
-          <t>Class 4 (TEL)</t>
+          <t>Class 5 (TEL)</t>
         </is>
       </c>
       <c r="G95" s="7" t="inlineStr">
         <is>
-          <t>Class 5 (TEL)</t>
+          <t>Class 3 (TEL)</t>
         </is>
       </c>
       <c r="H95" s="7" t="inlineStr"/>
@@ -3542,7 +3542,7 @@
       <c r="C96" s="7" t="inlineStr"/>
       <c r="D96" s="7" t="inlineStr">
         <is>
-          <t>Class 5 (TEL)</t>
+          <t>Class 4 (TEL)</t>
         </is>
       </c>
       <c r="E96" s="7" t="inlineStr">
@@ -3558,7 +3558,7 @@
       <c r="G96" s="7" t="inlineStr"/>
       <c r="H96" s="7" t="inlineStr">
         <is>
-          <t>Class 4 (TEL)</t>
+          <t>Class 5 (TEL)</t>
         </is>
       </c>
       <c r="I96" s="8" t="inlineStr">
@@ -3698,17 +3698,17 @@
       <c r="C100" s="7" t="inlineStr"/>
       <c r="D100" s="7" t="inlineStr">
         <is>
+          <t>Class 4 (TEL)</t>
+        </is>
+      </c>
+      <c r="E100" s="7" t="inlineStr">
+        <is>
           <t>Class 5 (TEL)</t>
         </is>
       </c>
-      <c r="E100" s="7" t="inlineStr">
+      <c r="F100" s="7" t="inlineStr">
         <is>
           <t>Class 3 (TEL)</t>
-        </is>
-      </c>
-      <c r="F100" s="7" t="inlineStr">
-        <is>
-          <t>Class 4 (TEL)</t>
         </is>
       </c>
       <c r="G100" s="7" t="inlineStr"/>
@@ -3867,7 +3867,7 @@
       </c>
       <c r="B106" s="7" t="inlineStr">
         <is>
-          <t>Class 5 (SOC)</t>
+          <t>Class 6 (SOC)</t>
         </is>
       </c>
       <c r="C106" s="7" t="inlineStr">
@@ -3878,7 +3878,7 @@
       <c r="D106" s="7" t="inlineStr"/>
       <c r="E106" s="7" t="inlineStr">
         <is>
-          <t>Class 4 (SOC)</t>
+          <t>Class 5 (SOC)</t>
         </is>
       </c>
       <c r="F106" s="7" t="inlineStr">
@@ -3889,7 +3889,7 @@
       <c r="G106" s="7" t="inlineStr"/>
       <c r="H106" s="7" t="inlineStr">
         <is>
-          <t>Class 6 (SOC)</t>
+          <t>Class 4 (SOC)</t>
         </is>
       </c>
       <c r="I106" s="8" t="inlineStr">
@@ -3984,28 +3984,28 @@
       </c>
       <c r="B109" s="7" t="inlineStr">
         <is>
-          <t>Class 6 (SOC)</t>
+          <t>Class 5 (SOC)</t>
         </is>
       </c>
       <c r="C109" s="7" t="inlineStr">
         <is>
-          <t>Class 5 (SOC)</t>
+          <t>Class 4 (SOC)</t>
         </is>
       </c>
       <c r="D109" s="7" t="inlineStr"/>
       <c r="E109" s="7" t="inlineStr">
         <is>
-          <t>Class 4 (SOC)</t>
+          <t>Class 3 (SOC)</t>
         </is>
       </c>
       <c r="F109" s="7" t="inlineStr">
         <is>
+          <t>Class 6 (SOC)</t>
+        </is>
+      </c>
+      <c r="G109" s="7" t="inlineStr">
+        <is>
           <t>Class 7 (SOC)</t>
-        </is>
-      </c>
-      <c r="G109" s="7" t="inlineStr">
-        <is>
-          <t>Class 3 (SOC)</t>
         </is>
       </c>
       <c r="H109" s="7" t="inlineStr"/>
@@ -4341,12 +4341,12 @@
       </c>
       <c r="C123" s="7" t="inlineStr">
         <is>
-          <t>Class 4 (EVS)</t>
+          <t>Class 6 (BIO)</t>
         </is>
       </c>
       <c r="D123" s="7" t="inlineStr">
         <is>
-          <t>Class 3 (EVS)</t>
+          <t>Class 3 (MATH)</t>
         </is>
       </c>
       <c r="E123" s="7" t="inlineStr"/>
@@ -4357,12 +4357,12 @@
       </c>
       <c r="G123" s="7" t="inlineStr">
         <is>
-          <t>Class 3 (MATH)</t>
+          <t>Class 3 (EVS)</t>
         </is>
       </c>
       <c r="H123" s="7" t="inlineStr">
         <is>
-          <t>Class 3 (MATH)</t>
+          <t>Class 4 (EVS)</t>
         </is>
       </c>
       <c r="I123" s="7" t="inlineStr"/>
@@ -4375,7 +4375,7 @@
       </c>
       <c r="B124" s="7" t="inlineStr">
         <is>
-          <t>Class 6 (BIO)</t>
+          <t>Class 4 (EVS)</t>
         </is>
       </c>
       <c r="C124" s="7" t="inlineStr">
@@ -4396,12 +4396,12 @@
       </c>
       <c r="G124" s="7" t="inlineStr">
         <is>
-          <t>Class 4 (EVS)</t>
+          <t>Class 3 (EVS)</t>
         </is>
       </c>
       <c r="H124" s="7" t="inlineStr">
         <is>
-          <t>Class 3 (EVS)</t>
+          <t>Class 3 (MATH)</t>
         </is>
       </c>
       <c r="I124" s="7" t="inlineStr"/>
@@ -4415,7 +4415,7 @@
       <c r="B125" s="7" t="inlineStr"/>
       <c r="C125" s="7" t="inlineStr">
         <is>
-          <t>Class 2 (EVS)</t>
+          <t>Class 2 (G.K)</t>
         </is>
       </c>
       <c r="D125" s="7" t="inlineStr">
@@ -4450,12 +4450,12 @@
       </c>
       <c r="C126" s="7" t="inlineStr">
         <is>
-          <t>Class 2 (G.K)</t>
+          <t>Class 2 (EVS)</t>
         </is>
       </c>
       <c r="D126" s="7" t="inlineStr">
         <is>
-          <t>Class 3 (EVS)</t>
+          <t>Class 3 (MATH)</t>
         </is>
       </c>
       <c r="E126" s="7" t="inlineStr"/>
@@ -4466,7 +4466,7 @@
       </c>
       <c r="G126" s="7" t="inlineStr">
         <is>
-          <t>Class 3 (MATH)</t>
+          <t>Class 3 (EVS)</t>
         </is>
       </c>
       <c r="H126" s="7" t="inlineStr">
@@ -4484,7 +4484,7 @@
       </c>
       <c r="B127" s="7" t="inlineStr">
         <is>
-          <t>Class 4 (EVS)</t>
+          <t>Class 6 (BIO)</t>
         </is>
       </c>
       <c r="C127" s="7" t="inlineStr">
@@ -4500,17 +4500,17 @@
       <c r="E127" s="7" t="inlineStr"/>
       <c r="F127" s="7" t="inlineStr">
         <is>
+          <t>Class 4 (EVS)</t>
+        </is>
+      </c>
+      <c r="G127" s="7" t="inlineStr">
+        <is>
+          <t>Class 3 (MATH)</t>
+        </is>
+      </c>
+      <c r="H127" s="7" t="inlineStr">
+        <is>
           <t>Class 3 (EVS)</t>
-        </is>
-      </c>
-      <c r="G127" s="7" t="inlineStr">
-        <is>
-          <t>Class 6 (BIO)</t>
-        </is>
-      </c>
-      <c r="H127" s="7" t="inlineStr">
-        <is>
-          <t>Class 3 (MATH)</t>
         </is>
       </c>
       <c r="I127" s="7" t="inlineStr"/>
@@ -4655,7 +4655,7 @@
       </c>
       <c r="B133" s="7" t="inlineStr">
         <is>
-          <t>Class 4 (HIN)</t>
+          <t>Class 5 (HIN)</t>
         </is>
       </c>
       <c r="C133" s="7" t="inlineStr">
@@ -4665,7 +4665,7 @@
       </c>
       <c r="D133" s="7" t="inlineStr">
         <is>
-          <t>Class 5 (HIN)</t>
+          <t>Class 6 (HIN)</t>
         </is>
       </c>
       <c r="E133" s="7" t="inlineStr">
@@ -4744,11 +4744,7 @@
           <t>Class 7 (HIN)</t>
         </is>
       </c>
-      <c r="G135" s="7" t="inlineStr">
-        <is>
-          <t>Class 6 (HIN)</t>
-        </is>
-      </c>
+      <c r="G135" s="7" t="inlineStr"/>
       <c r="H135" s="7" t="inlineStr"/>
       <c r="I135" s="8" t="inlineStr">
         <is>
@@ -4764,27 +4760,31 @@
       </c>
       <c r="B136" s="7" t="inlineStr">
         <is>
+          <t>Class 4 (HIN)</t>
+        </is>
+      </c>
+      <c r="C136" s="7" t="inlineStr">
+        <is>
           <t>Class 5 (HIN)</t>
         </is>
       </c>
-      <c r="C136" s="7" t="inlineStr">
+      <c r="D136" s="7" t="inlineStr">
+        <is>
+          <t>Class 3 (HIN)</t>
+        </is>
+      </c>
+      <c r="E136" s="7" t="inlineStr">
         <is>
           <t>Class 6 (HIN)</t>
-        </is>
-      </c>
-      <c r="D136" s="7" t="inlineStr">
-        <is>
-          <t>Class 3 (HIN)</t>
-        </is>
-      </c>
-      <c r="E136" s="7" t="inlineStr">
-        <is>
-          <t>Class 7 (HIN)</t>
         </is>
       </c>
       <c r="F136" s="7" t="inlineStr"/>
       <c r="G136" s="7" t="inlineStr"/>
-      <c r="H136" s="7" t="inlineStr"/>
+      <c r="H136" s="7" t="inlineStr">
+        <is>
+          <t>Class 7 (HIN)</t>
+        </is>
+      </c>
       <c r="I136" s="8" t="inlineStr">
         <is>
           <t>Class 4</t>
@@ -4879,13 +4879,13 @@
         </is>
       </c>
       <c r="B141" s="7" t="inlineStr"/>
-      <c r="C141" s="7" t="inlineStr">
-        <is>
-          <t>Class 9 (PHY)</t>
-        </is>
-      </c>
+      <c r="C141" s="7" t="inlineStr"/>
       <c r="D141" s="7" t="inlineStr"/>
-      <c r="E141" s="7" t="inlineStr"/>
+      <c r="E141" s="7" t="inlineStr">
+        <is>
+          <t>Class 10 (PHY)</t>
+        </is>
+      </c>
       <c r="F141" s="7" t="inlineStr"/>
       <c r="G141" s="7" t="inlineStr"/>
       <c r="H141" s="7" t="inlineStr"/>
@@ -4936,13 +4936,13 @@
         </is>
       </c>
       <c r="B144" s="7" t="inlineStr"/>
-      <c r="C144" s="7" t="inlineStr">
-        <is>
-          <t>Class 10 (PHY)</t>
-        </is>
-      </c>
+      <c r="C144" s="7" t="inlineStr"/>
       <c r="D144" s="7" t="inlineStr"/>
-      <c r="E144" s="7" t="inlineStr"/>
+      <c r="E144" s="7" t="inlineStr">
+        <is>
+          <t>Class 9 (PHY)</t>
+        </is>
+      </c>
       <c r="F144" s="7" t="inlineStr"/>
       <c r="G144" s="7" t="inlineStr"/>
       <c r="H144" s="7" t="inlineStr"/>
@@ -5037,7 +5037,7 @@
       </c>
       <c r="B149" s="7" t="inlineStr">
         <is>
-          <t>LKG (ENG)</t>
+          <t>LKG (EVS)</t>
         </is>
       </c>
       <c r="C149" s="7" t="inlineStr">
@@ -5106,7 +5106,7 @@
       <c r="G150" s="7" t="inlineStr"/>
       <c r="H150" s="7" t="inlineStr">
         <is>
-          <t>LKG (ENG)</t>
+          <t>LKG (MATH)</t>
         </is>
       </c>
       <c r="I150" s="8" t="inlineStr">
@@ -5138,7 +5138,7 @@
       </c>
       <c r="E151" s="7" t="inlineStr">
         <is>
-          <t>LKG (MATH)</t>
+          <t>LKG (ENG)</t>
         </is>
       </c>
       <c r="F151" s="7" t="inlineStr">
@@ -5170,12 +5170,12 @@
       </c>
       <c r="B152" s="7" t="inlineStr">
         <is>
+          <t>LKG (ENG)</t>
+        </is>
+      </c>
+      <c r="C152" s="7" t="inlineStr">
+        <is>
           <t>LKG (EVS)</t>
-        </is>
-      </c>
-      <c r="C152" s="7" t="inlineStr">
-        <is>
-          <t>LKG (ENG)</t>
         </is>
       </c>
       <c r="D152" s="7" t="inlineStr">
@@ -5213,7 +5213,7 @@
       </c>
       <c r="B153" s="7" t="inlineStr">
         <is>
-          <t>LKG (MATH)</t>
+          <t>LKG (EVS)</t>
         </is>
       </c>
       <c r="C153" s="7" t="inlineStr">
@@ -5260,7 +5260,7 @@
       </c>
       <c r="B154" s="7" t="inlineStr">
         <is>
-          <t>LKG (EVS)</t>
+          <t>LKG (ENG)</t>
         </is>
       </c>
       <c r="C154" s="7" t="inlineStr">
@@ -5270,7 +5270,7 @@
       </c>
       <c r="D154" s="7" t="inlineStr">
         <is>
-          <t>LKG (EVS)</t>
+          <t>LKG (MATH)</t>
         </is>
       </c>
       <c r="E154" s="7" t="inlineStr">
@@ -5593,22 +5593,22 @@
       </c>
       <c r="B167" s="7" t="inlineStr">
         <is>
+          <t>Class 1(B) (MATH)</t>
+        </is>
+      </c>
+      <c r="C167" s="7" t="inlineStr">
+        <is>
+          <t>Class 1(B) (MATH)</t>
+        </is>
+      </c>
+      <c r="D167" s="7" t="inlineStr">
+        <is>
+          <t>Class 1(B) (TEL)</t>
+        </is>
+      </c>
+      <c r="E167" s="7" t="inlineStr">
+        <is>
           <t>Class 1(B) (HIN)</t>
-        </is>
-      </c>
-      <c r="C167" s="7" t="inlineStr">
-        <is>
-          <t>Class 1(B) (MATH)</t>
-        </is>
-      </c>
-      <c r="D167" s="7" t="inlineStr">
-        <is>
-          <t>Class 1(B) (TEL)</t>
-        </is>
-      </c>
-      <c r="E167" s="7" t="inlineStr">
-        <is>
-          <t>Class 1(B) (MATH)</t>
         </is>
       </c>
       <c r="F167" s="7" t="inlineStr"/>
@@ -5941,7 +5941,7 @@
       <c r="B177" s="7" t="inlineStr"/>
       <c r="C177" s="7" t="inlineStr">
         <is>
-          <t>Class 6 (COMP)</t>
+          <t>Class 4 (COMP)</t>
         </is>
       </c>
       <c r="D177" s="7" t="inlineStr">
@@ -5982,7 +5982,11 @@
         </is>
       </c>
       <c r="F178" s="7" t="inlineStr"/>
-      <c r="G178" s="7" t="inlineStr"/>
+      <c r="G178" s="7" t="inlineStr">
+        <is>
+          <t>Class 1(A) (COMP)</t>
+        </is>
+      </c>
       <c r="H178" s="7" t="inlineStr"/>
       <c r="I178" s="7" t="inlineStr"/>
     </row>
@@ -6058,7 +6062,7 @@
       </c>
       <c r="D181" s="7" t="inlineStr">
         <is>
-          <t>Class 4 (COMP)</t>
+          <t>Class 6 (COMP)</t>
         </is>
       </c>
       <c r="E181" s="7" t="inlineStr">
@@ -6067,11 +6071,7 @@
         </is>
       </c>
       <c r="F181" s="7" t="inlineStr"/>
-      <c r="G181" s="7" t="inlineStr">
-        <is>
-          <t>Class 1(A) (COMP)</t>
-        </is>
-      </c>
+      <c r="G181" s="7" t="inlineStr"/>
       <c r="H181" s="7" t="inlineStr"/>
       <c r="I181" s="7" t="inlineStr"/>
     </row>
@@ -6150,12 +6150,12 @@
       <c r="F185" s="7" t="inlineStr"/>
       <c r="G185" s="7" t="inlineStr">
         <is>
-          <t>Class 2 (P.E.T)</t>
+          <t>Class 5 (P.E.T)</t>
         </is>
       </c>
       <c r="H185" s="7" t="inlineStr">
         <is>
-          <t>Class 6 (P.E.T)</t>
+          <t>Class 7 (P.E.T)</t>
         </is>
       </c>
       <c r="I185" s="7" t="inlineStr"/>
@@ -6196,7 +6196,7 @@
       <c r="F187" s="7" t="inlineStr"/>
       <c r="G187" s="7" t="inlineStr">
         <is>
-          <t>Class 3 (P.E.T)</t>
+          <t>Class 4 (P.E.T)</t>
         </is>
       </c>
       <c r="H187" s="7" t="inlineStr">
@@ -6238,7 +6238,7 @@
       <c r="F189" s="7" t="inlineStr"/>
       <c r="G189" s="7" t="inlineStr">
         <is>
-          <t>Class 2 (P.E.T)</t>
+          <t>Class 6 (P.E.T)</t>
         </is>
       </c>
       <c r="H189" s="7" t="inlineStr">
@@ -6261,12 +6261,12 @@
       <c r="F190" s="7" t="inlineStr"/>
       <c r="G190" s="7" t="inlineStr">
         <is>
-          <t>Class 7 (P.E.T)</t>
+          <t>Class 5 (P.E.T)</t>
         </is>
       </c>
       <c r="H190" s="7" t="inlineStr">
         <is>
-          <t>Class 5 (P.E.T)</t>
+          <t>Class 1(A) (P.E.T)</t>
         </is>
       </c>
       <c r="I190" s="7" t="inlineStr"/>
@@ -6578,7 +6578,7 @@
       <c r="C2" s="7" t="inlineStr">
         <is>
           <t>SHEKINA
-(ENG)</t>
+(EVS)</t>
         </is>
       </c>
       <c r="D2" s="7" t="inlineStr">
@@ -6590,19 +6590,19 @@
       <c r="E2" s="7" t="inlineStr">
         <is>
           <t>MAHA LAKSHMI
-(EVS)</t>
+(ENG)</t>
         </is>
       </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
           <t>CHANDRAKALA
+(TEL)</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>SURYA DEVI
 (MATH)</t>
-        </is>
-      </c>
-      <c r="G2" s="7" t="inlineStr">
-        <is>
-          <t>SURYA DEVI
-(HIN)</t>
         </is>
       </c>
       <c r="H2" s="7" t="inlineStr">
@@ -6686,7 +6686,7 @@
       <c r="F3" s="7" t="inlineStr">
         <is>
           <t>CHANDRAKALA
-(TEL)</t>
+(MATH)</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
@@ -6703,14 +6703,14 @@
       </c>
       <c r="I3" s="7" t="inlineStr">
         <is>
+          <t>N.NAVYA
+(ENG)</t>
+        </is>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
+        <is>
           <t>P.SATYAVENI
 (TEL)</t>
-        </is>
-      </c>
-      <c r="J3" s="7" t="inlineStr">
-        <is>
-          <t>N.NAVYA
-(ENG)</t>
         </is>
       </c>
       <c r="K3" s="7" t="inlineStr">
@@ -6870,7 +6870,7 @@
       <c r="G5" s="7" t="inlineStr">
         <is>
           <t>SURYA DEVI
-(MATH)</t>
+(HIN)</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
@@ -6887,14 +6887,14 @@
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
+          <t>N.NAVYA
+(ENG)</t>
+        </is>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
           <t>CHANDINI
 (MATH)</t>
-        </is>
-      </c>
-      <c r="K5" s="7" t="inlineStr">
-        <is>
-          <t>N.NAVYA
-(ENG)</t>
         </is>
       </c>
       <c r="L5" s="7" t="inlineStr">
@@ -6974,14 +6974,14 @@
       </c>
       <c r="J6" s="7" t="inlineStr">
         <is>
+          <t>CHANDINI
+(MATH)</t>
+        </is>
+      </c>
+      <c r="K6" s="7" t="inlineStr">
+        <is>
           <t>P.SATYAVENI
 (TEL)</t>
-        </is>
-      </c>
-      <c r="K6" s="7" t="inlineStr">
-        <is>
-          <t>CHANDINI
-(MATH)</t>
         </is>
       </c>
       <c r="L6" s="7" t="inlineStr">
@@ -7058,8 +7058,8 @@
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>N.NAVYA
-(ENG)</t>
+          <t>P.SATYAVENI
+(TEL)</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
@@ -7070,8 +7070,8 @@
       </c>
       <c r="K7" s="7" t="inlineStr">
         <is>
-          <t>P.SATYAVENI
-(TEL)</t>
+          <t>P.E.T Instructor
+(P.E.T)</t>
         </is>
       </c>
       <c r="L7" s="7" t="inlineStr">
@@ -7083,7 +7083,7 @@
       <c r="M7" s="7" t="inlineStr">
         <is>
           <t>K.ESWAR
-(PHY)</t>
+(CHEM)</t>
         </is>
       </c>
       <c r="N7" s="7" t="inlineStr">
@@ -7154,26 +7154,26 @@
       </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
+          <t>N.NAVYA
+(ENG)</t>
+        </is>
+      </c>
+      <c r="K8" s="7" t="inlineStr">
+        <is>
+          <t>R.KAMALA
+(SOC)</t>
+        </is>
+      </c>
+      <c r="L8" s="7" t="inlineStr">
+        <is>
+          <t>K.ESWAR
+(CHEM)</t>
+        </is>
+      </c>
+      <c r="M8" s="7" t="inlineStr">
+        <is>
           <t>P.E.T Instructor
 (P.E.T)</t>
-        </is>
-      </c>
-      <c r="K8" s="7" t="inlineStr">
-        <is>
-          <t>R.KAMALA
-(SOC)</t>
-        </is>
-      </c>
-      <c r="L8" s="7" t="inlineStr">
-        <is>
-          <t>P.E.T Instructor
-(P.E.T)</t>
-        </is>
-      </c>
-      <c r="M8" s="7" t="inlineStr">
-        <is>
-          <t>K.ESWAR
-(CHEM)</t>
         </is>
       </c>
       <c r="N8" s="7" t="inlineStr">
@@ -7395,7 +7395,7 @@
       <c r="D11" s="7" t="inlineStr">
         <is>
           <t>BIJILI
-(ENG)</t>
+(MATH)</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -7407,7 +7407,7 @@
       <c r="F11" s="7" t="inlineStr">
         <is>
           <t>CHANDRAKALA
-(HIN)</t>
+(MATH)</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -7430,8 +7430,8 @@
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>S.GAYATHRI
-(EVS)</t>
+          <t>VINAY
+(COMP)</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
@@ -7442,14 +7442,14 @@
       </c>
       <c r="L11" s="7" t="inlineStr">
         <is>
-          <t>VINAY
-(COMP)</t>
+          <t>S.GAYATHRI
+(BIO)</t>
         </is>
       </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
           <t>K.ESWAR
-(G.K)</t>
+(PHY)</t>
         </is>
       </c>
       <c r="N11" s="7" t="inlineStr">
@@ -7458,10 +7458,9 @@
 (MATH)</t>
         </is>
       </c>
-      <c r="O11" s="7" t="inlineStr">
-        <is>
-          <t>SAIRAM
-(PHY)</t>
+      <c r="O11" s="12" t="inlineStr">
+        <is>
+          <t>Recreation</t>
         </is>
       </c>
       <c r="P11" s="7" t="inlineStr">
@@ -7515,19 +7514,19 @@
       <c r="I12" s="7" t="inlineStr">
         <is>
           <t>S.GAYATHRI
-(EVS)</t>
+(MATH)</t>
         </is>
       </c>
       <c r="J12" s="7" t="inlineStr">
+        <is>
+          <t>P.SATYAVENI
+(TEL)</t>
+        </is>
+      </c>
+      <c r="K12" s="7" t="inlineStr">
         <is>
           <t>N.NAVYA
 (ENG)</t>
-        </is>
-      </c>
-      <c r="K12" s="7" t="inlineStr">
-        <is>
-          <t>P.SATYAVENI
-(TEL)</t>
         </is>
       </c>
       <c r="L12" s="7" t="inlineStr">
@@ -7643,9 +7642,10 @@
 (TEL)</t>
         </is>
       </c>
-      <c r="P13" s="12" t="inlineStr">
-        <is>
-          <t>Recreation</t>
+      <c r="P13" s="7" t="inlineStr">
+        <is>
+          <t>SAIRAM
+(PHY)</t>
         </is>
       </c>
     </row>
@@ -7675,7 +7675,7 @@
       <c r="F14" s="7" t="inlineStr">
         <is>
           <t>CHANDRAKALA
-(MATH)</t>
+(G.K)</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
@@ -7758,8 +7758,8 @@
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>MAHA LAKSHMI
-(ENG)</t>
+          <t>P.E.T Instructor
+(P.E.T)</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
@@ -7783,7 +7783,7 @@
       <c r="I15" s="7" t="inlineStr">
         <is>
           <t>S.GAYATHRI
-(MATH)</t>
+(EVS)</t>
         </is>
       </c>
       <c r="J15" s="7" t="inlineStr">
@@ -7807,7 +7807,7 @@
       <c r="M15" s="7" t="inlineStr">
         <is>
           <t>K.ESWAR
-(CHEM)</t>
+(G.K)</t>
         </is>
       </c>
       <c r="N15" s="7" t="inlineStr">
@@ -7837,7 +7837,7 @@
       <c r="C16" s="7" t="inlineStr">
         <is>
           <t>SHEKINA
-(ENG)</t>
+(MATH)</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
@@ -7872,20 +7872,20 @@
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
+          <t>P.E.T Instructor
+(P.E.T)</t>
+        </is>
+      </c>
+      <c r="J16" s="7" t="inlineStr">
+        <is>
           <t>S.GAYATHRI
-(MATH)</t>
-        </is>
-      </c>
-      <c r="J16" s="7" t="inlineStr">
+(EVS)</t>
+        </is>
+      </c>
+      <c r="K16" s="7" t="inlineStr">
         <is>
           <t>P.SATYAVENI
 (TEL)</t>
-        </is>
-      </c>
-      <c r="K16" s="7" t="inlineStr">
-        <is>
-          <t>P.E.T Instructor
-(P.E.T)</t>
         </is>
       </c>
       <c r="L16" s="7" t="inlineStr">
@@ -8064,20 +8064,20 @@
       </c>
       <c r="J18" s="7" t="inlineStr">
         <is>
+          <t>S.GAYATHRI
+(EVS)</t>
+        </is>
+      </c>
+      <c r="K18" s="7" t="inlineStr">
+        <is>
           <t>SAI KEERTHI
 (HIN)</t>
         </is>
       </c>
-      <c r="K18" s="7" t="inlineStr">
+      <c r="L18" s="7" t="inlineStr">
         <is>
           <t>R.KAMALA
 (SOC)</t>
-        </is>
-      </c>
-      <c r="L18" s="7" t="inlineStr">
-        <is>
-          <t>S.GAYATHRI
-(BIO)</t>
         </is>
       </c>
       <c r="M18" s="7" t="inlineStr">
@@ -8175,9 +8175,10 @@
 (SOC)</t>
         </is>
       </c>
-      <c r="N19" s="12" t="inlineStr">
-        <is>
-          <t>Recreation</t>
+      <c r="N19" s="7" t="inlineStr">
+        <is>
+          <t>CHALAPATHI
+(BIO)</t>
         </is>
       </c>
       <c r="O19" s="7" t="inlineStr">
@@ -8248,14 +8249,14 @@
       </c>
       <c r="K20" s="7" t="inlineStr">
         <is>
+          <t>CHANDINI
+(MATH)</t>
+        </is>
+      </c>
+      <c r="L20" s="7" t="inlineStr">
+        <is>
           <t>SAI KEERTHI
 (HIN)</t>
-        </is>
-      </c>
-      <c r="L20" s="7" t="inlineStr">
-        <is>
-          <t>CHANDINI
-(MATH)</t>
         </is>
       </c>
       <c r="M20" s="7" t="inlineStr">
@@ -8291,7 +8292,7 @@
       <c r="C21" s="7" t="inlineStr">
         <is>
           <t>SHEKINA
-(MATH)</t>
+(ENG)</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
@@ -8332,14 +8333,14 @@
       </c>
       <c r="J21" s="7" t="inlineStr">
         <is>
+          <t>CHANDINI
+(MATH)</t>
+        </is>
+      </c>
+      <c r="K21" s="7" t="inlineStr">
+        <is>
           <t>R.KAMALA
 (SOC)</t>
-        </is>
-      </c>
-      <c r="K21" s="7" t="inlineStr">
-        <is>
-          <t>CHANDINI
-(MATH)</t>
         </is>
       </c>
       <c r="L21" s="7" t="inlineStr">
@@ -8486,8 +8487,8 @@
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>CHANDRAKALA
-(G.K)</t>
+          <t>VINAY
+(COMP)</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -8498,20 +8499,20 @@
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
+          <t>CHANDRAKALA
+(MATH)</t>
+        </is>
+      </c>
+      <c r="I23" s="7" t="inlineStr">
+        <is>
+          <t>S.GAYATHRI
+(EVS)</t>
+        </is>
+      </c>
+      <c r="J23" s="7" t="inlineStr">
+        <is>
           <t>P.E.T Instructor
 (P.E.T)</t>
-        </is>
-      </c>
-      <c r="I23" s="7" t="inlineStr">
-        <is>
-          <t>P.E.T Instructor
-(P.E.T)</t>
-        </is>
-      </c>
-      <c r="J23" s="7" t="inlineStr">
-        <is>
-          <t>S.GAYATHRI
-(EVS)</t>
         </is>
       </c>
       <c r="K23" s="7" t="inlineStr">
@@ -8595,31 +8596,31 @@
       <c r="I24" s="7" t="inlineStr">
         <is>
           <t>S.GAYATHRI
-(EVS)</t>
+(MATH)</t>
         </is>
       </c>
       <c r="J24" s="7" t="inlineStr">
+        <is>
+          <t>R.KAMALA
+(SOC)</t>
+        </is>
+      </c>
+      <c r="K24" s="7" t="inlineStr">
+        <is>
+          <t>N.NAVYA
+(ENG)</t>
+        </is>
+      </c>
+      <c r="L24" s="7" t="inlineStr">
         <is>
           <t>CHANDINI
 (MATH)</t>
         </is>
       </c>
-      <c r="K24" s="7" t="inlineStr">
-        <is>
-          <t>N.NAVYA
-(ENG)</t>
-        </is>
-      </c>
-      <c r="L24" s="7" t="inlineStr">
-        <is>
-          <t>R.KAMALA
-(SOC)</t>
-        </is>
-      </c>
       <c r="M24" s="7" t="inlineStr">
         <is>
           <t>K.ESWAR
-(PHY)</t>
+(CHEM)</t>
         </is>
       </c>
       <c r="N24" s="7" t="inlineStr">
@@ -8745,7 +8746,7 @@
       <c r="C26" s="7" t="inlineStr">
         <is>
           <t>SHEKINA
-(EVS)</t>
+(ENG)</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
@@ -8763,7 +8764,7 @@
       <c r="F26" s="7" t="inlineStr">
         <is>
           <t>CHANDRAKALA
-(MATH)</t>
+(EVS)</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
@@ -8835,7 +8836,7 @@
       <c r="C27" s="7" t="inlineStr">
         <is>
           <t>SHEKINA
-(ENG)</t>
+(EVS)</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
@@ -8865,7 +8866,7 @@
       <c r="H27" s="7" t="inlineStr">
         <is>
           <t>S.GAYATHRI
-(EVS)</t>
+(G.K)</t>
         </is>
       </c>
       <c r="I27" s="7" t="inlineStr">
@@ -8889,7 +8890,7 @@
       <c r="L27" s="7" t="inlineStr">
         <is>
           <t>K.ESWAR
-(CHEM)</t>
+(PHY)</t>
         </is>
       </c>
       <c r="M27" s="7" t="inlineStr">
@@ -9120,7 +9121,7 @@
       <c r="F30" s="7" t="inlineStr">
         <is>
           <t>CHANDRAKALA
-(EVS)</t>
+(MATH)</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
@@ -9468,7 +9469,7 @@
       <c r="C34" s="7" t="inlineStr">
         <is>
           <t>SHEKINA
-(MATH)</t>
+(EVS)</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
@@ -9588,7 +9589,7 @@
       <c r="H35" s="7" t="inlineStr">
         <is>
           <t>S.GAYATHRI
-(G.K)</t>
+(EVS)</t>
         </is>
       </c>
       <c r="I35" s="7" t="inlineStr">
@@ -9621,10 +9622,9 @@
 (MATH)</t>
         </is>
       </c>
-      <c r="N35" s="7" t="inlineStr">
-        <is>
-          <t>CHALAPATHI
-(BIO)</t>
+      <c r="N35" s="12" t="inlineStr">
+        <is>
+          <t>Recreation</t>
         </is>
       </c>
       <c r="O35" s="7" t="inlineStr">
@@ -9633,10 +9633,9 @@
 (ENG)</t>
         </is>
       </c>
-      <c r="P35" s="7" t="inlineStr">
-        <is>
-          <t>SAIRAM
-(PHY)</t>
+      <c r="P35" s="12" t="inlineStr">
+        <is>
+          <t>Recreation</t>
         </is>
       </c>
     </row>
@@ -9684,7 +9683,7 @@
       <c r="I36" s="7" t="inlineStr">
         <is>
           <t>S.GAYATHRI
-(EVS)</t>
+(MATH)</t>
         </is>
       </c>
       <c r="J36" s="7" t="inlineStr">
@@ -9807,9 +9806,10 @@
 (MATH)</t>
         </is>
       </c>
-      <c r="O37" s="12" t="inlineStr">
-        <is>
-          <t>Recreation</t>
+      <c r="O37" s="7" t="inlineStr">
+        <is>
+          <t>SAIRAM
+(PHY)</t>
         </is>
       </c>
       <c r="P37" s="12" t="inlineStr">
@@ -9927,50 +9927,50 @@
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
+          <t>MAHA LAKSHMI
+(EVS)</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>CHANDRAKALA
+(HIN)</t>
+        </is>
+      </c>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>SURYA DEVI
+(HIN)</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
           <t>P.E.T Instructor
 (P.E.T)</t>
         </is>
       </c>
-      <c r="F39" s="7" t="inlineStr">
-        <is>
-          <t>CHANDRAKALA
+      <c r="I39" s="7" t="inlineStr">
+        <is>
+          <t>S.GAYATHRI
+(EVS)</t>
+        </is>
+      </c>
+      <c r="J39" s="7" t="inlineStr">
+        <is>
+          <t>CHANDINI
+(MATH)</t>
+        </is>
+      </c>
+      <c r="K39" s="7" t="inlineStr">
+        <is>
+          <t>N.NAVYA
 (ENG)</t>
         </is>
       </c>
-      <c r="G39" s="7" t="inlineStr">
-        <is>
-          <t>SURYA DEVI
-(HIN)</t>
-        </is>
-      </c>
-      <c r="H39" s="7" t="inlineStr">
+      <c r="L39" s="7" t="inlineStr">
         <is>
           <t>P.E.T Instructor
 (P.E.T)</t>
-        </is>
-      </c>
-      <c r="I39" s="7" t="inlineStr">
-        <is>
-          <t>S.GAYATHRI
-(MATH)</t>
-        </is>
-      </c>
-      <c r="J39" s="7" t="inlineStr">
-        <is>
-          <t>CHANDINI
-(MATH)</t>
-        </is>
-      </c>
-      <c r="K39" s="7" t="inlineStr">
-        <is>
-          <t>N.NAVYA
-(ENG)</t>
-        </is>
-      </c>
-      <c r="L39" s="7" t="inlineStr">
-        <is>
-          <t>SAI KEERTHI
-(HIN)</t>
         </is>
       </c>
       <c r="M39" s="7" t="inlineStr">
@@ -10192,7 +10192,7 @@
       <c r="C42" s="7" t="inlineStr">
         <is>
           <t>SHEKINA
-(EVS)</t>
+(ENG)</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
@@ -10210,7 +10210,7 @@
       <c r="F42" s="7" t="inlineStr">
         <is>
           <t>CHANDRAKALA
-(TEL)</t>
+(ENG)</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
@@ -10233,20 +10233,20 @@
       </c>
       <c r="J42" s="7" t="inlineStr">
         <is>
-          <t>S.GAYATHRI
-(EVS)</t>
-        </is>
-      </c>
-      <c r="K42" s="7" t="inlineStr">
-        <is>
           <t>SAI KEERTHI
 (HIN)</t>
         </is>
       </c>
-      <c r="L42" s="7" t="inlineStr">
+      <c r="K42" s="7" t="inlineStr">
         <is>
           <t>R.KAMALA
 (SOC)</t>
+        </is>
+      </c>
+      <c r="L42" s="7" t="inlineStr">
+        <is>
+          <t>S.GAYATHRI
+(BIO)</t>
         </is>
       </c>
       <c r="M42" s="7" t="inlineStr">
@@ -10323,22 +10323,22 @@
       </c>
       <c r="J43" s="7" t="inlineStr">
         <is>
+          <t>R.KAMALA
+(SOC)</t>
+        </is>
+      </c>
+      <c r="K43" s="7" t="inlineStr">
+        <is>
+          <t>SAI KEERTHI
+(HIN)</t>
+        </is>
+      </c>
+      <c r="L43" s="7" t="inlineStr">
+        <is>
           <t>CHANDINI
 (MATH)</t>
         </is>
       </c>
-      <c r="K43" s="7" t="inlineStr">
-        <is>
-          <t>R.KAMALA
-(SOC)</t>
-        </is>
-      </c>
-      <c r="L43" s="7" t="inlineStr">
-        <is>
-          <t>SAI KEERTHI
-(HIN)</t>
-        </is>
-      </c>
       <c r="M43" s="7" t="inlineStr">
         <is>
           <t>D.SUMANI
@@ -10351,9 +10351,10 @@
 (COMP)</t>
         </is>
       </c>
-      <c r="O43" s="12" t="inlineStr">
-        <is>
-          <t>Recreation</t>
+      <c r="O43" s="7" t="inlineStr">
+        <is>
+          <t>CHALAPATHI
+(BIO)</t>
         </is>
       </c>
       <c r="P43" s="7" t="inlineStr">
@@ -10371,7 +10372,7 @@
       <c r="C44" s="7" t="inlineStr">
         <is>
           <t>SHEKINA
-(EVS)</t>
+(MATH)</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
@@ -10412,22 +10413,22 @@
       </c>
       <c r="J44" s="7" t="inlineStr">
         <is>
+          <t>P.SATYAVENI
+(TEL)</t>
+        </is>
+      </c>
+      <c r="K44" s="7" t="inlineStr">
+        <is>
+          <t>N.NAVYA
+(ENG)</t>
+        </is>
+      </c>
+      <c r="L44" s="7" t="inlineStr">
+        <is>
           <t>VINAY
 (COMP)</t>
         </is>
       </c>
-      <c r="K44" s="7" t="inlineStr">
-        <is>
-          <t>P.SATYAVENI
-(TEL)</t>
-        </is>
-      </c>
-      <c r="L44" s="7" t="inlineStr">
-        <is>
-          <t>N.NAVYA
-(ENG)</t>
-        </is>
-      </c>
       <c r="M44" s="7" t="inlineStr">
         <is>
           <t>K.ESWAR
@@ -10440,10 +10441,9 @@
 (TEL)</t>
         </is>
       </c>
-      <c r="O44" s="7" t="inlineStr">
-        <is>
-          <t>CHALAPATHI
-(BIO)</t>
+      <c r="O44" s="12" t="inlineStr">
+        <is>
+          <t>Recreation</t>
         </is>
       </c>
       <c r="P44" s="7" t="inlineStr">
@@ -10479,7 +10479,7 @@
       <c r="F45" s="7" t="inlineStr">
         <is>
           <t>CHANDRAKALA
-(EVS)</t>
+(TEL)</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
@@ -10496,32 +10496,32 @@
       </c>
       <c r="I45" s="7" t="inlineStr">
         <is>
+          <t>R.KAMALA
+(SOC)</t>
+        </is>
+      </c>
+      <c r="J45" s="7" t="inlineStr">
+        <is>
+          <t>CHANDINI
+(MATH)</t>
+        </is>
+      </c>
+      <c r="K45" s="7" t="inlineStr">
+        <is>
           <t>P.SATYAVENI
 (TEL)</t>
         </is>
       </c>
-      <c r="J45" s="7" t="inlineStr">
-        <is>
-          <t>R.KAMALA
-(SOC)</t>
-        </is>
-      </c>
-      <c r="K45" s="7" t="inlineStr">
-        <is>
-          <t>CHANDINI
-(MATH)</t>
-        </is>
-      </c>
       <c r="L45" s="7" t="inlineStr">
+        <is>
+          <t>SAI KEERTHI
+(HIN)</t>
+        </is>
+      </c>
+      <c r="M45" s="7" t="inlineStr">
         <is>
           <t>K.ESWAR
 (PHY)</t>
-        </is>
-      </c>
-      <c r="M45" s="7" t="inlineStr">
-        <is>
-          <t>SAI KEERTHI
-(HIN)</t>
         </is>
       </c>
       <c r="N45" s="12" t="inlineStr">
@@ -10556,7 +10556,7 @@
       <c r="D46" s="7" t="inlineStr">
         <is>
           <t>BIJILI
-(MATH)</t>
+(ENG)</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
@@ -10585,16 +10585,16 @@
       </c>
       <c r="I46" s="7" t="inlineStr">
         <is>
+          <t>P.SATYAVENI
+(TEL)</t>
+        </is>
+      </c>
+      <c r="J46" s="7" t="inlineStr">
+        <is>
           <t>S.GAYATHRI
 (EVS)</t>
         </is>
       </c>
-      <c r="J46" s="7" t="inlineStr">
-        <is>
-          <t>P.SATYAVENI
-(TEL)</t>
-        </is>
-      </c>
       <c r="K46" s="7" t="inlineStr">
         <is>
           <t>K.ESWAR
@@ -10603,14 +10603,14 @@
       </c>
       <c r="L46" s="7" t="inlineStr">
         <is>
+          <t>R.KAMALA
+(SOC)</t>
+        </is>
+      </c>
+      <c r="M46" s="7" t="inlineStr">
+        <is>
           <t>M.LALITHA
 (TEL)</t>
-        </is>
-      </c>
-      <c r="M46" s="7" t="inlineStr">
-        <is>
-          <t>R.KAMALA
-(SOC)</t>
         </is>
       </c>
       <c r="N46" s="7" t="inlineStr">
@@ -10657,8 +10657,8 @@
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>VINAY
-(COMP)</t>
+          <t>CHANDRAKALA
+(EVS)</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
@@ -10669,38 +10669,38 @@
       </c>
       <c r="H47" s="7" t="inlineStr">
         <is>
-          <t>CHANDRAKALA
+          <t>P.E.T Instructor
+(P.E.T)</t>
+        </is>
+      </c>
+      <c r="I47" s="7" t="inlineStr">
+        <is>
+          <t>S.GAYATHRI
 (MATH)</t>
         </is>
       </c>
-      <c r="I47" s="7" t="inlineStr">
+      <c r="J47" s="7" t="inlineStr">
+        <is>
+          <t>P.E.T Instructor
+(P.E.T)</t>
+        </is>
+      </c>
+      <c r="K47" s="7" t="inlineStr">
+        <is>
+          <t>P.E.T Instructor
+(P.E.T)</t>
+        </is>
+      </c>
+      <c r="L47" s="7" t="inlineStr">
+        <is>
+          <t>N.NAVYA
+(ENG)</t>
+        </is>
+      </c>
+      <c r="M47" s="7" t="inlineStr">
         <is>
           <t>R.KAMALA
 (SOC)</t>
-        </is>
-      </c>
-      <c r="J47" s="7" t="inlineStr">
-        <is>
-          <t>P.E.T Instructor
-(P.E.T)</t>
-        </is>
-      </c>
-      <c r="K47" s="7" t="inlineStr">
-        <is>
-          <t>N.NAVYA
-(ENG)</t>
-        </is>
-      </c>
-      <c r="L47" s="7" t="inlineStr">
-        <is>
-          <t>S.GAYATHRI
-(BIO)</t>
-        </is>
-      </c>
-      <c r="M47" s="7" t="inlineStr">
-        <is>
-          <t>P.E.T Instructor
-(P.E.T)</t>
         </is>
       </c>
       <c r="N47" s="7" t="inlineStr">
@@ -10766,7 +10766,7 @@
       <c r="I48" s="7" t="inlineStr">
         <is>
           <t>S.GAYATHRI
-(MATH)</t>
+(EVS)</t>
         </is>
       </c>
       <c r="J48" s="7" t="inlineStr">
@@ -10777,20 +10777,20 @@
       </c>
       <c r="K48" s="7" t="inlineStr">
         <is>
-          <t>P.E.T Instructor
-(P.E.T)</t>
-        </is>
-      </c>
-      <c r="L48" s="7" t="inlineStr">
-        <is>
           <t>CHANDINI
 (MATH)</t>
         </is>
       </c>
-      <c r="M48" s="7" t="inlineStr">
+      <c r="L48" s="7" t="inlineStr">
         <is>
           <t>M.LALITHA
 (TEL)</t>
+        </is>
+      </c>
+      <c r="M48" s="7" t="inlineStr">
+        <is>
+          <t>SAI KEERTHI
+(HIN)</t>
         </is>
       </c>
       <c r="N48" s="7" t="inlineStr">

</xml_diff>